<commit_message>
risoluzione outliers, estensione analisi dati
</commit_message>
<xml_diff>
--- a/exploratory_data_analysis/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
+++ b/exploratory_data_analysis/risultati/correlazioni_dispersioni/matrice_correlazione.xlsx
@@ -545,64 +545,64 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4216116756900395</v>
+        <v>0.4107699984382805</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.04475880514129424</v>
+        <v>-0.04493181898450962</v>
       </c>
       <c r="E2" t="n">
-        <v>0.05340572670807206</v>
+        <v>0.06269640499425402</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.05678692972028783</v>
+        <v>-0.05716260179848934</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.04694186872321313</v>
+        <v>-0.03423136919851529</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5201352381463509</v>
+        <v>0.5330536100799442</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5253530561870094</v>
+        <v>0.4795555932535001</v>
       </c>
       <c r="J2" t="n">
-        <v>0.003937791249886274</v>
+        <v>0.05552533860160565</v>
       </c>
       <c r="K2" t="n">
-        <v>0.06126020035590456</v>
+        <v>0.04203575712036502</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6122801074946496</v>
+        <v>0.5718754782474768</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.09366965241541637</v>
+        <v>-0.08777209459367555</v>
       </c>
       <c r="N2" t="n">
-        <v>0.003067045524870239</v>
+        <v>0.01123505744624869</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1087800313330247</v>
+        <v>0.1078863661900788</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.07425680499168422</v>
+        <v>-0.06583491728536627</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.05974297865797865</v>
+        <v>-0.06048329863432983</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.004376195880742525</v>
+        <v>-0.004563937708362182</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3772023668696086</v>
+        <v>0.343799723740856</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.02089704747108574</v>
+        <v>-0.02070391312107526</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.05557134264104221</v>
+        <v>-0.06365188075385719</v>
       </c>
       <c r="V2" t="n">
-        <v>0.3375184569016842</v>
+        <v>0.3518101614444146</v>
       </c>
     </row>
     <row r="3">
@@ -612,67 +612,67 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4216116756900395</v>
+        <v>0.4107699984382805</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1779934158126077</v>
+        <v>0.1828761076342559</v>
       </c>
       <c r="E3" t="n">
-        <v>0.104935069600181</v>
+        <v>0.1055009350893324</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.06277091374462798</v>
+        <v>-0.06016475804327828</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.01642376737729592</v>
+        <v>-0.01220457914885962</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1227774323467498</v>
+        <v>0.1184393218019089</v>
       </c>
       <c r="I3" t="n">
-        <v>0.722448144599707</v>
+        <v>0.7433945007005733</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.01159045770967008</v>
+        <v>-0.01467818331302639</v>
       </c>
       <c r="K3" t="n">
-        <v>0.02932680395634131</v>
+        <v>0.02268010090802798</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3331236982107779</v>
+        <v>0.3114196436117996</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02813261583997162</v>
+        <v>0.03325489258525646</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.02758803212797382</v>
+        <v>-0.02665276217754529</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.05131346189181413</v>
+        <v>-0.05607939130695003</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.00784680351638507</v>
+        <v>-0.003559187584605272</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.02219220950974682</v>
+        <v>0.02438662303138875</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.03989168788205612</v>
+        <v>-0.03977922569002665</v>
       </c>
       <c r="S3" t="n">
-        <v>0.8807892386975859</v>
+        <v>0.8784996283862436</v>
       </c>
       <c r="T3" t="n">
-        <v>0.149234342922977</v>
+        <v>0.1535198516506619</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.04916562457079351</v>
+        <v>-0.04977467624260799</v>
       </c>
       <c r="V3" t="n">
-        <v>0.4346824417956081</v>
+        <v>0.4320471878952345</v>
       </c>
     </row>
     <row r="4">
@@ -682,67 +682,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.04475880514129424</v>
+        <v>-0.04493181898450962</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1779934158126077</v>
+        <v>0.1828761076342559</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1327836512630097</v>
+        <v>-0.1456033772007568</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.04353970960727233</v>
+        <v>-0.0386444791826261</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004580041004354343</v>
+        <v>-0.002882600313852715</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.01806591717440596</v>
+        <v>-0.04035047138908179</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1541990774896825</v>
+        <v>0.1650976047058155</v>
       </c>
       <c r="J4" t="n">
-        <v>0.007223111395267638</v>
+        <v>0.0103976195557689</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.01364399222591401</v>
+        <v>-0.01270287605049416</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.02221600837727774</v>
+        <v>-0.02018417697929265</v>
       </c>
       <c r="M4" t="n">
-        <v>0.077080548865487</v>
+        <v>0.0655937961450038</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.06944708618472717</v>
+        <v>-0.07118238355349395</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.08380134218004327</v>
+        <v>-0.07517130136672991</v>
       </c>
       <c r="P4" t="n">
-        <v>0.06409294834383399</v>
+        <v>0.04971217140480956</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.06253882406071057</v>
+        <v>0.05391174584077664</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.06002228659102011</v>
+        <v>-0.05600307509311708</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1888840749157984</v>
+        <v>0.1948503726085103</v>
       </c>
       <c r="T4" t="n">
-        <v>0.6274001289591388</v>
+        <v>0.6205228536659727</v>
       </c>
       <c r="U4" t="n">
-        <v>0.05125722192573615</v>
+        <v>0.05034897530674703</v>
       </c>
       <c r="V4" t="n">
-        <v>-0.07078340294831489</v>
+        <v>-0.06815082952630173</v>
       </c>
     </row>
     <row r="5">
@@ -752,67 +752,67 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05340572670807206</v>
+        <v>0.06269640499425402</v>
       </c>
       <c r="C5" t="n">
-        <v>0.104935069600181</v>
+        <v>0.1055009350893324</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1327836512630097</v>
+        <v>-0.1456033772007568</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.07109200201510901</v>
+        <v>-0.07804394797776851</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1121660353341882</v>
+        <v>0.1102022605438197</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0009788642935270619</v>
+        <v>-0.1041258286466655</v>
       </c>
       <c r="I5" t="n">
-        <v>0.004582624283223379</v>
+        <v>0.01491342987048542</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.1068916439266058</v>
+        <v>-0.3768984365207781</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.03992448149446571</v>
+        <v>-0.03986707901417107</v>
       </c>
       <c r="L5" t="n">
-        <v>0.01507093830297792</v>
+        <v>0.01634077623741607</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3578683979053901</v>
+        <v>0.3540270520001535</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4961855462666429</v>
+        <v>0.4983228475601495</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.3093946497529023</v>
+        <v>-0.306025012526734</v>
       </c>
       <c r="P5" t="n">
-        <v>0.375330788215232</v>
+        <v>0.3708186626299486</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.007211201451642502</v>
+        <v>-0.01352937325599825</v>
       </c>
       <c r="R5" t="n">
-        <v>-0.1623671261839348</v>
+        <v>-0.1605073527495656</v>
       </c>
       <c r="S5" t="n">
-        <v>0.04729208238050727</v>
+        <v>0.04773325963785345</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.1266281700883653</v>
+        <v>-0.1356547459399113</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.2169260343682781</v>
+        <v>-0.2163144824324924</v>
       </c>
       <c r="V5" t="n">
-        <v>0.253330498132152</v>
+        <v>0.253129699496333</v>
       </c>
     </row>
     <row r="6">
@@ -822,67 +822,67 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.05678692972028783</v>
+        <v>-0.05716260179848934</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.06277091374462798</v>
+        <v>-0.06016475804327828</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.04353970960727233</v>
+        <v>-0.0386444791826261</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.07109200201510901</v>
+        <v>-0.07804394797776851</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.3781312858705676</v>
+        <v>-0.3904905114205633</v>
       </c>
       <c r="H6" t="n">
-        <v>0.007839297613693053</v>
+        <v>0.2564129871631383</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.01564201164827849</v>
+        <v>-0.002750206817131486</v>
       </c>
       <c r="J6" t="n">
-        <v>0.002767420027318275</v>
+        <v>0.3333822472966903</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.008007868839107689</v>
+        <v>-0.006835690923019978</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.04626193499149509</v>
+        <v>-0.04430470311093584</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.3454058303393051</v>
+        <v>-0.3479335926520875</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.3398366335316781</v>
+        <v>-0.3521962682310001</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2730748644624182</v>
+        <v>0.2711843017700764</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.3991671199733859</v>
+        <v>-0.4065422351426727</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.2060898167069142</v>
+        <v>-0.1972055437614216</v>
       </c>
       <c r="R6" t="n">
-        <v>0.2234441401857156</v>
+        <v>0.2178107841466263</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.02599354691460453</v>
+        <v>-0.0223324398989442</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.02048834059667011</v>
+        <v>-0.01827652646098101</v>
       </c>
       <c r="U6" t="n">
-        <v>0.1340290143796559</v>
+        <v>0.1321416088647652</v>
       </c>
       <c r="V6" t="n">
-        <v>0.111836435019094</v>
+        <v>0.1146312326963627</v>
       </c>
     </row>
     <row r="7">
@@ -892,67 +892,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.04694186872321313</v>
+        <v>-0.03423136919851529</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.01642376737729592</v>
+        <v>-0.01220457914885962</v>
       </c>
       <c r="D7" t="n">
-        <v>0.004580041004354343</v>
+        <v>-0.002882600313852715</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1121660353341882</v>
+        <v>0.1102022605438197</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.3781312858705676</v>
+        <v>-0.3904905114205633</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.05455308160020825</v>
+        <v>-0.236939642745481</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.07296202496460717</v>
+        <v>-0.07103610072442132</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0440200129214556</v>
+        <v>-0.3740466364527545</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0180196108202791</v>
+        <v>0.02023879606983839</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.006248086443202955</v>
+        <v>0.003329540816539707</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4068862829846087</v>
+        <v>0.4057565423170194</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4039175919529504</v>
+        <v>0.4041245965119598</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.3150274522952745</v>
+        <v>-0.3131078921006562</v>
       </c>
       <c r="P7" t="n">
-        <v>0.4891773034526148</v>
+        <v>0.4891957791185136</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1335168876693346</v>
+        <v>0.1299171412307018</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.1061921092020066</v>
+        <v>-0.1044963156843923</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.03840406540807877</v>
+        <v>-0.03380422176561212</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.0002980273419669136</v>
+        <v>-0.004680557464565218</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.0818831125453803</v>
+        <v>-0.08563968501436756</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.1055822790731904</v>
+        <v>-0.1022749987092068</v>
       </c>
     </row>
     <row r="8">
@@ -962,67 +962,67 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.5201352381463509</v>
+        <v>0.5330536100799442</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1227774323467498</v>
+        <v>0.1184393218019089</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.01806591717440596</v>
+        <v>-0.04035047138908179</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0009788642935270619</v>
+        <v>-0.1041258286466655</v>
       </c>
       <c r="F8" t="n">
-        <v>0.007839297613693053</v>
+        <v>0.2564129871631383</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.05455308160020825</v>
+        <v>-0.236939642745481</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1547998283547365</v>
+        <v>0.2838063135303538</v>
       </c>
       <c r="J8" t="n">
-        <v>0.002202906225295654</v>
+        <v>0.3015311196530265</v>
       </c>
       <c r="K8" t="n">
-        <v>0.01671382285621353</v>
+        <v>0.02787838947075083</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2394087033883915</v>
+        <v>0.1479122709797734</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.09136070877678065</v>
+        <v>-0.3944119310105226</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.03198016661505865</v>
+        <v>-0.2477174010630281</v>
       </c>
       <c r="O8" t="n">
-        <v>0.09959937189403691</v>
+        <v>0.3872246228969416</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.07534957719361846</v>
+        <v>-0.3634503929322483</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.05990985252367347</v>
+        <v>-0.2013418226373828</v>
       </c>
       <c r="R8" t="n">
-        <v>0.02985654676729521</v>
+        <v>0.1212480898397185</v>
       </c>
       <c r="S8" t="n">
-        <v>0.1343149376418389</v>
+        <v>0.1507081158631169</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.008999636590506099</v>
+        <v>-0.01906854572490414</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0115070127290727</v>
+        <v>0.01917596765100124</v>
       </c>
       <c r="V8" t="n">
-        <v>0.1774593700166999</v>
+        <v>0.183694839367484</v>
       </c>
     </row>
     <row r="9">
@@ -1032,67 +1032,67 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.5253530561870094</v>
+        <v>0.4795555932535001</v>
       </c>
       <c r="C9" t="n">
-        <v>0.722448144599707</v>
+        <v>0.7433945007005733</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1541990774896825</v>
+        <v>0.1650976047058155</v>
       </c>
       <c r="E9" t="n">
-        <v>0.004582624283223379</v>
+        <v>0.01491342987048542</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.01564201164827849</v>
+        <v>-0.002750206817131486</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.07296202496460717</v>
+        <v>-0.07103610072442132</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1547998283547365</v>
+        <v>0.2838063135303538</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1002567884994365</v>
+        <v>0.1497566126786699</v>
       </c>
       <c r="K9" t="n">
-        <v>0.04806806631643538</v>
+        <v>0.03745777803860717</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2847912257757358</v>
+        <v>0.242481671902537</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.07412555028207493</v>
+        <v>-0.07171309602886784</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.09341252538709487</v>
+        <v>-0.0958382681315406</v>
       </c>
       <c r="O9" t="n">
-        <v>0.05006308977836382</v>
+        <v>0.04324460764811788</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.0962627071668308</v>
+        <v>-0.09963798373698418</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.01242901942121015</v>
+        <v>-0.01300879597066246</v>
       </c>
       <c r="R9" t="n">
-        <v>-0.0133511012102141</v>
+        <v>-0.01208090011615016</v>
       </c>
       <c r="S9" t="n">
-        <v>0.7885101632054529</v>
+        <v>0.7968916784100238</v>
       </c>
       <c r="T9" t="n">
-        <v>0.173075175565739</v>
+        <v>0.1486566072293661</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.0157186637594478</v>
+        <v>-0.02161929935831005</v>
       </c>
       <c r="V9" t="n">
-        <v>0.3429567748683054</v>
+        <v>0.352215120246655</v>
       </c>
     </row>
     <row r="10">
@@ -1102,67 +1102,67 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.003937791249886274</v>
+        <v>0.05552533860160565</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.01159045770967008</v>
+        <v>-0.01467818331302639</v>
       </c>
       <c r="D10" t="n">
-        <v>0.007223111395267638</v>
+        <v>0.0103976195557689</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1068916439266058</v>
+        <v>-0.3768984365207781</v>
       </c>
       <c r="F10" t="n">
-        <v>0.002767420027318275</v>
+        <v>0.3333822472966903</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0440200129214556</v>
+        <v>-0.3740466364527545</v>
       </c>
       <c r="H10" t="n">
-        <v>0.002202906225295654</v>
+        <v>0.3015311196530265</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1002567884994365</v>
+        <v>0.1497566126786699</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0004232297979541761</v>
+        <v>0.02054100481888916</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0003019608166179558</v>
+        <v>0.006614441028997577</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.05232536252482686</v>
+        <v>-0.6970097388231949</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.09113045045995571</v>
+        <v>-0.4742064939306004</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0541846475359171</v>
+        <v>0.6306626213264016</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.04100934745247311</v>
+        <v>-0.6919283241009963</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.0007129725155011026</v>
+        <v>-0.4202658561250584</v>
       </c>
       <c r="R10" t="n">
-        <v>0.01752882526649929</v>
+        <v>0.3147057019203685</v>
       </c>
       <c r="S10" t="n">
-        <v>0.005309815336748252</v>
+        <v>0.02345826157931083</v>
       </c>
       <c r="T10" t="n">
-        <v>0.2718152208080674</v>
+        <v>0.03937048345836729</v>
       </c>
       <c r="U10" t="n">
-        <v>0.04041876648741743</v>
+        <v>0.03307085724047992</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.01778810985546364</v>
+        <v>0.04130398301374855</v>
       </c>
     </row>
     <row r="11">
@@ -1172,67 +1172,67 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.06126020035590456</v>
+        <v>0.04203575712036502</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02932680395634131</v>
+        <v>0.02268010090802798</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.01364399222591401</v>
+        <v>-0.01270287605049416</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.03992448149446571</v>
+        <v>-0.03986707901417107</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.008007868839107689</v>
+        <v>-0.006835690923019978</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0180196108202791</v>
+        <v>0.02023879606983839</v>
       </c>
       <c r="H11" t="n">
-        <v>0.01671382285621353</v>
+        <v>0.02787838947075083</v>
       </c>
       <c r="I11" t="n">
-        <v>0.04806806631643538</v>
+        <v>0.03745777803860717</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0004232297979541761</v>
+        <v>0.02054100481888916</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.03770769642340872</v>
+        <v>0.02500066842630837</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.01754791561086857</v>
+        <v>-0.01543672175437564</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.05097929286907681</v>
+        <v>-0.05067343872034188</v>
       </c>
       <c r="O11" t="n">
-        <v>0.004939476008869307</v>
+        <v>0.00309427038783579</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.02827710635366739</v>
+        <v>-0.02620403761486678</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.03861923343226006</v>
+        <v>0.04004131284992362</v>
       </c>
       <c r="R11" t="n">
-        <v>-0.00706704334137514</v>
+        <v>-0.007095745571080414</v>
       </c>
       <c r="S11" t="n">
-        <v>0.0297843172675414</v>
+        <v>0.02162411386714837</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.00802334891561363</v>
+        <v>-0.007587630743704312</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.02432575730776702</v>
+        <v>-0.0246404985988846</v>
       </c>
       <c r="V11" t="n">
-        <v>0.03781692223053876</v>
+        <v>0.03477680669374338</v>
       </c>
     </row>
     <row r="12">
@@ -1242,67 +1242,67 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.6122801074946496</v>
+        <v>0.5718754782474768</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3331236982107779</v>
+        <v>0.3114196436117996</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.02221600837727774</v>
+        <v>-0.02018417697929265</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01507093830297792</v>
+        <v>0.01634077623741607</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.04626193499149509</v>
+        <v>-0.04430470311093584</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.006248086443202955</v>
+        <v>0.003329540816539707</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2394087033883915</v>
+        <v>0.1479122709797734</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2847912257757358</v>
+        <v>0.242481671902537</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0003019608166179558</v>
+        <v>0.006614441028997577</v>
       </c>
       <c r="K12" t="n">
-        <v>0.03770769642340872</v>
+        <v>0.02500066842630837</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.03919827694340727</v>
+        <v>-0.03115892015530013</v>
       </c>
       <c r="N12" t="n">
-        <v>0.05546104686238104</v>
+        <v>0.06183327030033405</v>
       </c>
       <c r="O12" t="n">
-        <v>0.04013635395803889</v>
+        <v>0.03352265137596259</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.0391281456129627</v>
+        <v>-0.03131859752700795</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.04723142431962738</v>
+        <v>-0.04566218407760123</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.00132689129944614</v>
+        <v>-0.0009689161339465025</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2649880336774942</v>
+        <v>0.2321299472214066</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.01106111394547585</v>
+        <v>-0.01005568225578336</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.05047990442057526</v>
+        <v>-0.05268009763488148</v>
       </c>
       <c r="V12" t="n">
-        <v>0.2390508181251627</v>
+        <v>0.2317545416880752</v>
       </c>
     </row>
     <row r="13">
@@ -1312,67 +1312,67 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.09366965241541637</v>
+        <v>-0.08777209459367555</v>
       </c>
       <c r="C13" t="n">
-        <v>0.02813261583997162</v>
+        <v>0.03325489258525646</v>
       </c>
       <c r="D13" t="n">
-        <v>0.077080548865487</v>
+        <v>0.0655937961450038</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3578683979053901</v>
+        <v>0.3540270520001535</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.3454058303393051</v>
+        <v>-0.3479335926520875</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4068862829846087</v>
+        <v>0.4057565423170194</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.09136070877678065</v>
+        <v>-0.3944119310105226</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.07412555028207493</v>
+        <v>-0.07171309602886784</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.05232536252482686</v>
+        <v>-0.6970097388231949</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.01754791561086857</v>
+        <v>-0.01543672175437564</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.03919827694340727</v>
+        <v>-0.03115892015530013</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>0.4499789179418643</v>
+        <v>0.4521348448097253</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.9580512166292018</v>
+        <v>-0.9576207327943297</v>
       </c>
       <c r="P13" t="n">
-        <v>0.9355127139247841</v>
+        <v>0.9345539800872096</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.6725953612431936</v>
+        <v>0.6679941812612148</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.4566626251383287</v>
+        <v>-0.452280205443447</v>
       </c>
       <c r="S13" t="n">
-        <v>0.004799001326287505</v>
+        <v>0.01082501261331815</v>
       </c>
       <c r="T13" t="n">
-        <v>0.05198338768730814</v>
+        <v>0.04567630412457926</v>
       </c>
       <c r="U13" t="n">
-        <v>0.01449977015368358</v>
+        <v>0.01960986702368907</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.08588168720750974</v>
+        <v>-0.08355244279345746</v>
       </c>
     </row>
     <row r="14">
@@ -1382,67 +1382,67 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.003067045524870239</v>
+        <v>0.01123505744624869</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.02758803212797382</v>
+        <v>-0.02665276217754529</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.06944708618472717</v>
+        <v>-0.07118238355349395</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4961855462666429</v>
+        <v>0.4983228475601495</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.3398366335316781</v>
+        <v>-0.3521962682310001</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4039175919529504</v>
+        <v>0.4041245965119598</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.03198016661505865</v>
+        <v>-0.2477174010630281</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.09341252538709487</v>
+        <v>-0.0958382681315406</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.09113045045995571</v>
+        <v>-0.4742064939306004</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.05097929286907681</v>
+        <v>-0.05067343872034188</v>
       </c>
       <c r="L14" t="n">
-        <v>0.05546104686238104</v>
+        <v>0.06183327030033405</v>
       </c>
       <c r="M14" t="n">
-        <v>0.4499789179418643</v>
+        <v>0.4521348448097253</v>
       </c>
       <c r="N14" t="n">
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>-0.3521643357791112</v>
+        <v>-0.3521419990598738</v>
       </c>
       <c r="P14" t="n">
-        <v>0.5206682742873963</v>
+        <v>0.5252630020747105</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.09749921138377071</v>
+        <v>-0.1039784790349556</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.1358411520883878</v>
+        <v>-0.1339912246788807</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.06255450987651977</v>
+        <v>-0.06245179780370444</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.07917322739223173</v>
+        <v>-0.08316973521712806</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.1569889386490672</v>
+        <v>-0.1548597192434937</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.03683063246752379</v>
+        <v>-0.0384583162273814</v>
       </c>
     </row>
     <row r="15">
@@ -1452,67 +1452,67 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1087800313330247</v>
+        <v>0.1078863661900788</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.05131346189181413</v>
+        <v>-0.05607939130695003</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.08380134218004327</v>
+        <v>-0.07517130136672991</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.3093946497529023</v>
+        <v>-0.306025012526734</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2730748644624182</v>
+        <v>0.2711843017700764</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.3150274522952745</v>
+        <v>-0.3131078921006562</v>
       </c>
       <c r="H15" t="n">
-        <v>0.09959937189403691</v>
+        <v>0.3872246228969416</v>
       </c>
       <c r="I15" t="n">
-        <v>0.05006308977836382</v>
+        <v>0.04324460764811788</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0541846475359171</v>
+        <v>0.6306626213264016</v>
       </c>
       <c r="K15" t="n">
-        <v>0.004939476008869307</v>
+        <v>0.00309427038783579</v>
       </c>
       <c r="L15" t="n">
-        <v>0.04013635395803889</v>
+        <v>0.03352265137596259</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.9580512166292018</v>
+        <v>-0.9576207327943297</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.3521643357791112</v>
+        <v>-0.3521419990598738</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>
       </c>
       <c r="P15" t="n">
-        <v>-0.800456456636485</v>
+        <v>-0.7979812445226</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.7007481459261141</v>
+        <v>-0.6966610021879354</v>
       </c>
       <c r="R15" t="n">
-        <v>0.4973849426082247</v>
+        <v>0.4930277056705943</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.03016676939244723</v>
+        <v>-0.03584663720280416</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.06203324567102053</v>
+        <v>-0.05763686799343103</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.02992854744645928</v>
+        <v>-0.03585292053059695</v>
       </c>
       <c r="V15" t="n">
-        <v>0.02880193135588411</v>
+        <v>0.02636361835787374</v>
       </c>
     </row>
     <row r="16">
@@ -1522,67 +1522,67 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.07425680499168422</v>
+        <v>-0.06583491728536627</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.00784680351638507</v>
+        <v>-0.003559187584605272</v>
       </c>
       <c r="D16" t="n">
-        <v>0.06409294834383399</v>
+        <v>0.04971217140480956</v>
       </c>
       <c r="E16" t="n">
-        <v>0.375330788215232</v>
+        <v>0.3708186626299486</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.3991671199733859</v>
+        <v>-0.4065422351426727</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4891773034526148</v>
+        <v>0.4891957791185136</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.07534957719361846</v>
+        <v>-0.3634503929322483</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.0962627071668308</v>
+        <v>-0.09963798373698418</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.04100934745247311</v>
+        <v>-0.6919283241009963</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.02827710635366739</v>
+        <v>-0.02620403761486678</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.0391281456129627</v>
+        <v>-0.03131859752700795</v>
       </c>
       <c r="M16" t="n">
-        <v>0.9355127139247841</v>
+        <v>0.9345539800872096</v>
       </c>
       <c r="N16" t="n">
-        <v>0.5206682742873963</v>
+        <v>0.5252630020747105</v>
       </c>
       <c r="O16" t="n">
-        <v>-0.800456456636485</v>
+        <v>-0.7979812445226</v>
       </c>
       <c r="P16" t="n">
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.5545299422721117</v>
+        <v>0.5483232232155537</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.3570189515794582</v>
+        <v>-0.3522493765375893</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.03209503799845873</v>
+        <v>-0.02713192621841959</v>
       </c>
       <c r="T16" t="n">
-        <v>0.03496540579652683</v>
+        <v>0.02653631913926469</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.009003189511974638</v>
+        <v>-0.005743644569526904</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.1563063448729051</v>
+        <v>-0.154659456228817</v>
       </c>
     </row>
     <row r="17">
@@ -1592,67 +1592,67 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.05974297865797865</v>
+        <v>-0.06048329863432983</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02219220950974682</v>
+        <v>0.02438662303138875</v>
       </c>
       <c r="D17" t="n">
-        <v>0.06253882406071057</v>
+        <v>0.05391174584077664</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.007211201451642502</v>
+        <v>-0.01352937325599825</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.2060898167069142</v>
+        <v>-0.1972055437614216</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1335168876693346</v>
+        <v>0.1299171412307018</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.05990985252367347</v>
+        <v>-0.2013418226373828</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.01242901942121015</v>
+        <v>-0.01300879597066246</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0007129725155011026</v>
+        <v>-0.4202658561250584</v>
       </c>
       <c r="K17" t="n">
-        <v>0.03861923343226006</v>
+        <v>0.04004131284992362</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.04723142431962738</v>
+        <v>-0.04566218407760123</v>
       </c>
       <c r="M17" t="n">
-        <v>0.6725953612431936</v>
+        <v>0.6679941812612148</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.09749921138377071</v>
+        <v>-0.1039784790349556</v>
       </c>
       <c r="O17" t="n">
-        <v>-0.7007481459261141</v>
+        <v>-0.6966610021879354</v>
       </c>
       <c r="P17" t="n">
-        <v>0.5545299422721117</v>
+        <v>0.5483232232155537</v>
       </c>
       <c r="Q17" t="n">
         <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.4894004645416619</v>
+        <v>-0.4843575067089396</v>
       </c>
       <c r="S17" t="n">
-        <v>0.02885324227809394</v>
+        <v>0.03183282181000241</v>
       </c>
       <c r="T17" t="n">
-        <v>0.06797792727324876</v>
+        <v>0.06444122965699417</v>
       </c>
       <c r="U17" t="n">
-        <v>0.1179512595118699</v>
+        <v>0.1265143597509155</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.08377084597072579</v>
+        <v>-0.08165043816949583</v>
       </c>
     </row>
     <row r="18">
@@ -1662,67 +1662,67 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.004376195880742525</v>
+        <v>-0.004563937708362182</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.03989168788205612</v>
+        <v>-0.03977922569002665</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.06002228659102011</v>
+        <v>-0.05600307509311708</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.1623671261839348</v>
+        <v>-0.1605073527495656</v>
       </c>
       <c r="F18" t="n">
-        <v>0.2234441401857156</v>
+        <v>0.2178107841466263</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.1061921092020066</v>
+        <v>-0.1044963156843923</v>
       </c>
       <c r="H18" t="n">
-        <v>0.02985654676729521</v>
+        <v>0.1212480898397185</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.0133511012102141</v>
+        <v>-0.01208090011615016</v>
       </c>
       <c r="J18" t="n">
-        <v>0.01752882526649929</v>
+        <v>0.3147057019203685</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.00706704334137514</v>
+        <v>-0.007095745571080414</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.00132689129944614</v>
+        <v>-0.0009689161339465025</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.4566626251383287</v>
+        <v>-0.452280205443447</v>
       </c>
       <c r="N18" t="n">
-        <v>-0.1358411520883878</v>
+        <v>-0.1339912246788807</v>
       </c>
       <c r="O18" t="n">
-        <v>0.4973849426082247</v>
+        <v>0.4930277056705943</v>
       </c>
       <c r="P18" t="n">
-        <v>-0.3570189515794582</v>
+        <v>-0.3522493765375893</v>
       </c>
       <c r="Q18" t="n">
-        <v>-0.4894004645416619</v>
+        <v>-0.4843575067089396</v>
       </c>
       <c r="R18" t="n">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.03267103785982577</v>
+        <v>-0.03271394137719008</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.04188605077938152</v>
+        <v>-0.03990516193969423</v>
       </c>
       <c r="U18" t="n">
-        <v>0.03923372681035635</v>
+        <v>0.03535199604169725</v>
       </c>
       <c r="V18" t="n">
-        <v>0.01563485934282179</v>
+        <v>0.01554740783267842</v>
       </c>
     </row>
     <row r="19">
@@ -1732,67 +1732,67 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.3772023668696086</v>
+        <v>0.343799723740856</v>
       </c>
       <c r="C19" t="n">
-        <v>0.8807892386975859</v>
+        <v>0.8784996283862436</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1888840749157984</v>
+        <v>0.1948503726085103</v>
       </c>
       <c r="E19" t="n">
-        <v>0.04729208238050727</v>
+        <v>0.04773325963785345</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.02599354691460453</v>
+        <v>-0.0223324398989442</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.03840406540807877</v>
+        <v>-0.03380422176561212</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1343149376418389</v>
+        <v>0.1507081158631169</v>
       </c>
       <c r="I19" t="n">
-        <v>0.7885101632054529</v>
+        <v>0.7968916784100238</v>
       </c>
       <c r="J19" t="n">
-        <v>0.005309815336748252</v>
+        <v>0.02345826157931083</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0297843172675414</v>
+        <v>0.02162411386714837</v>
       </c>
       <c r="L19" t="n">
-        <v>0.2649880336774942</v>
+        <v>0.2321299472214066</v>
       </c>
       <c r="M19" t="n">
-        <v>0.004799001326287505</v>
+        <v>0.01082501261331815</v>
       </c>
       <c r="N19" t="n">
-        <v>-0.06255450987651977</v>
+        <v>-0.06245179780370444</v>
       </c>
       <c r="O19" t="n">
-        <v>-0.03016676939244723</v>
+        <v>-0.03584663720280416</v>
       </c>
       <c r="P19" t="n">
-        <v>-0.03209503799845873</v>
+        <v>-0.02713192621841959</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.02885324227809394</v>
+        <v>0.03183282181000241</v>
       </c>
       <c r="R19" t="n">
-        <v>-0.03267103785982577</v>
+        <v>-0.03271394137719008</v>
       </c>
       <c r="S19" t="n">
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>0.2455969487423447</v>
+        <v>0.2516912498979388</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.02377380836842913</v>
+        <v>-0.02427257907927612</v>
       </c>
       <c r="V19" t="n">
-        <v>0.3587726988534073</v>
+        <v>0.3552104268138176</v>
       </c>
     </row>
     <row r="20">
@@ -1802,67 +1802,67 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.02089704747108574</v>
+        <v>-0.02070391312107526</v>
       </c>
       <c r="C20" t="n">
-        <v>0.149234342922977</v>
+        <v>0.1535198516506619</v>
       </c>
       <c r="D20" t="n">
-        <v>0.6274001289591388</v>
+        <v>0.6205228536659727</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1266281700883653</v>
+        <v>-0.1356547459399113</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.02048834059667011</v>
+        <v>-0.01827652646098101</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0002980273419669136</v>
+        <v>-0.004680557464565218</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.008999636590506099</v>
+        <v>-0.01906854572490414</v>
       </c>
       <c r="I20" t="n">
-        <v>0.173075175565739</v>
+        <v>0.1486566072293661</v>
       </c>
       <c r="J20" t="n">
-        <v>0.2718152208080674</v>
+        <v>0.03937048345836729</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.00802334891561363</v>
+        <v>-0.007587630743704312</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.01106111394547585</v>
+        <v>-0.01005568225578336</v>
       </c>
       <c r="M20" t="n">
-        <v>0.05198338768730814</v>
+        <v>0.04567630412457926</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.07917322739223173</v>
+        <v>-0.08316973521712806</v>
       </c>
       <c r="O20" t="n">
-        <v>-0.06203324567102053</v>
+        <v>-0.05763686799343103</v>
       </c>
       <c r="P20" t="n">
-        <v>0.03496540579652683</v>
+        <v>0.02653631913926469</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.06797792727324876</v>
+        <v>0.06444122965699417</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.04188605077938152</v>
+        <v>-0.03990516193969423</v>
       </c>
       <c r="S20" t="n">
-        <v>0.2455969487423447</v>
+        <v>0.2516912498979388</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
       </c>
       <c r="U20" t="n">
-        <v>0.02576470963131629</v>
+        <v>0.02333780367300154</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.04095615075635482</v>
+        <v>-0.03850305260236042</v>
       </c>
     </row>
     <row r="21">
@@ -1872,67 +1872,67 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.05557134264104221</v>
+        <v>-0.06365188075385719</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.04916562457079351</v>
+        <v>-0.04977467624260799</v>
       </c>
       <c r="D21" t="n">
-        <v>0.05125722192573615</v>
+        <v>0.05034897530674703</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.2169260343682781</v>
+        <v>-0.2163144824324924</v>
       </c>
       <c r="F21" t="n">
-        <v>0.1340290143796559</v>
+        <v>0.1321416088647652</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.0818831125453803</v>
+        <v>-0.08563968501436756</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0115070127290727</v>
+        <v>0.01917596765100124</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.0157186637594478</v>
+        <v>-0.02161929935831005</v>
       </c>
       <c r="J21" t="n">
-        <v>0.04041876648741743</v>
+        <v>0.03307085724047992</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.02432575730776702</v>
+        <v>-0.0246404985988846</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.05047990442057526</v>
+        <v>-0.05268009763488148</v>
       </c>
       <c r="M21" t="n">
-        <v>0.01449977015368358</v>
+        <v>0.01960986702368907</v>
       </c>
       <c r="N21" t="n">
-        <v>-0.1569889386490672</v>
+        <v>-0.1548597192434937</v>
       </c>
       <c r="O21" t="n">
-        <v>-0.02992854744645928</v>
+        <v>-0.03585292053059695</v>
       </c>
       <c r="P21" t="n">
-        <v>-0.009003189511974638</v>
+        <v>-0.005743644569526904</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.1179512595118699</v>
+        <v>0.1265143597509155</v>
       </c>
       <c r="R21" t="n">
-        <v>0.03923372681035635</v>
+        <v>0.03535199604169725</v>
       </c>
       <c r="S21" t="n">
-        <v>-0.02377380836842913</v>
+        <v>-0.02427257907927612</v>
       </c>
       <c r="T21" t="n">
-        <v>0.02576470963131629</v>
+        <v>0.02333780367300154</v>
       </c>
       <c r="U21" t="n">
         <v>1</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.0835880288472004</v>
+        <v>-0.08018534865245608</v>
       </c>
     </row>
     <row r="22">
@@ -1942,64 +1942,64 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.3375184569016842</v>
+        <v>0.3518101614444146</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4346824417956081</v>
+        <v>0.4320471878952345</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.07078340294831489</v>
+        <v>-0.06815082952630173</v>
       </c>
       <c r="E22" t="n">
-        <v>0.253330498132152</v>
+        <v>0.253129699496333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.111836435019094</v>
+        <v>0.1146312326963627</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.1055822790731904</v>
+        <v>-0.1022749987092068</v>
       </c>
       <c r="H22" t="n">
-        <v>0.1774593700166999</v>
+        <v>0.183694839367484</v>
       </c>
       <c r="I22" t="n">
-        <v>0.3429567748683054</v>
+        <v>0.352215120246655</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.01778810985546364</v>
+        <v>0.04130398301374855</v>
       </c>
       <c r="K22" t="n">
-        <v>0.03781692223053876</v>
+        <v>0.03477680669374338</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2390508181251627</v>
+        <v>0.2317545416880752</v>
       </c>
       <c r="M22" t="n">
-        <v>-0.08588168720750974</v>
+        <v>-0.08355244279345746</v>
       </c>
       <c r="N22" t="n">
-        <v>-0.03683063246752379</v>
+        <v>-0.0384583162273814</v>
       </c>
       <c r="O22" t="n">
-        <v>0.02880193135588411</v>
+        <v>0.02636361835787374</v>
       </c>
       <c r="P22" t="n">
-        <v>-0.1563063448729051</v>
+        <v>-0.154659456228817</v>
       </c>
       <c r="Q22" t="n">
-        <v>-0.08377084597072579</v>
+        <v>-0.08165043816949583</v>
       </c>
       <c r="R22" t="n">
-        <v>0.01563485934282179</v>
+        <v>0.01554740783267842</v>
       </c>
       <c r="S22" t="n">
-        <v>0.3587726988534073</v>
+        <v>0.3552104268138176</v>
       </c>
       <c r="T22" t="n">
-        <v>-0.04095615075635482</v>
+        <v>-0.03850305260236042</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.0835880288472004</v>
+        <v>-0.08018534865245608</v>
       </c>
       <c r="V22" t="n">
         <v>1</v>

</xml_diff>